<commit_message>
Record the real Progress capture and the StoreKit rerun.
Both devices opened Progress. Annual cancel and expiry passed. Monthly expireSubscription threw a StoreKit test error.

Co-authored-by: armctay85 <armctay85@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/audit/2026-10-15/findings.xlsx
+++ b/docs/audit/2026-10-15/findings.xlsx
@@ -499,6 +499,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -567,7 +568,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>https://github.com/armctay85/FitMunch/actions/runs/38673394433</t>
+          <t>https://github.com/armctay85/FitMunch/actions/runs/38673394433 and follow-up https://github.com/armctay85/FitMunch/actions/runs/38703638103</t>
         </is>
       </c>
     </row>
@@ -603,7 +604,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>SKTestSession on the 6.9in simulator. fitmunch_weekly absent. Monthly and annual purchase, 14-day trial, entitlement, and restore passed. Monthly cancel passed. Annual cancel failed (willAutoRenew stayed true). Expiry failed for both (state stayed subscribed).</t>
+          <t>SKTestSession rerun on the 6.9in simulator (run 38703638103). Test catalog displayPrice was $19.99 monthly and $149.99 annual, currency AUD. fitmunch_weekly absent. Annual cancel and expiry passed (willAutoRenew false, RenewalState expired, entitlement cleared). Monthly cancel passed. Monthly expireSubscription threw SKTestErrorDomain Code=6. That is a StoreKit Testing limit, not app code.</t>
         </is>
       </c>
     </row>
@@ -619,6 +620,7 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
@@ -636,7 +638,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="16">
@@ -646,9 +648,10 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>7</v>
-      </c>
-    </row>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17"/>
     <row r="18" ht="48" customHeight="1">
       <c r="A18" t="inlineStr">
         <is>
@@ -657,7 +660,7 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Auth error (session-expired copy on a bad password). Today offline (empty meal line hidden, PR 153). Settings about on 6.9in (March 2025, PR 154). Progress (screen never opened).</t>
+          <t>Auth error (session-expired copy on a bad password). Today offline (empty meal line hidden, PR 153). Settings about on 6.9in (March 2025, PR 154).</t>
         </is>
       </c>
     </row>
@@ -2545,18 +2548,20 @@
       </c>
       <c r="D47" s="8" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="E47" s="6" t="inlineStr">
         <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="F47" s="6" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F47" s="6" t="n">
+        <v>7</v>
+      </c>
       <c r="G47" s="6" t="inlineStr">
         <is>
-          <t>Progress never opened. The screenshot matches Me scrolled to Data. The Progress row sits at the top and was offscreen after the About scroll.</t>
+          <t>Follow-up opened Progress from Me. Date Range, Statistics, and the empty meal copy are on screen.</t>
         </is>
       </c>
       <c r="H47" s="6" t="inlineStr">
@@ -4383,18 +4388,20 @@
       </c>
       <c r="D93" s="8" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="E93" s="6" t="inlineStr">
         <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="F93" s="6" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F93" s="6" t="n">
+        <v>7</v>
+      </c>
       <c r="G93" s="6" t="inlineStr">
         <is>
-          <t>Progress never opened. The screenshot matches Me scrolled to Data. The Progress row sits at the top and was offscreen after the About scroll.</t>
+          <t>Follow-up opened Progress from Me. Date Range, Statistics, and the empty meal copy are on screen.</t>
         </is>
       </c>
       <c r="H93" s="6" t="inlineStr">

</xml_diff>